<commit_message>
feat: busca entrada NF-e, vínculo XML, wizard e edição cliente PDV
Adiciona busca livre e filtros avançados na lista de notas; melhora auto-vínculo
por cProd/descrição e backfill histórico; corrige parcelas editáveis e avanço do
wizard; permite editar cliente no PDV; atualiza dados de cashback pendentes.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/dados/saldo_cashback.xlsx
+++ b/dados/saldo_cashback.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c79cfebefc6519e2/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c79cfebefc6519e2/Documentos/GitHub/agro-consulta/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{4ABA237C-F67F-4712-B371-8BDA0358A578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F01805C-59B5-4642-999B-D514FE88F1B3}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{4ABA237C-F67F-4712-B371-8BDA0358A578}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EED82269-77E7-4899-A4FA-947A9CB0AE82}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{EA56A08E-E1C3-4A31-881E-2FD8F7AC7A97}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$B$1068</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3276,10 +3279,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3317,7 +3324,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3423,7 +3430,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3565,7 +3572,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3575,6 +3582,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{342CB184-3FA6-4140-8743-3A005F6668F9}">
   <dimension ref="A1:B1068"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="45.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.4609375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
@@ -4621,7 +4632,7 @@
         <v>131</v>
       </c>
       <c r="B131">
-        <v>6.38</v>
+        <v>0.38</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.4">
@@ -4733,7 +4744,7 @@
         <v>145</v>
       </c>
       <c r="B145">
-        <v>0.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.4">
@@ -5253,7 +5264,7 @@
         <v>210</v>
       </c>
       <c r="B210">
-        <v>6.72</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211" spans="1:2" x14ac:dyDescent="0.4">
@@ -12121,6 +12132,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1068" xr:uid="{342CB184-3FA6-4140-8743-3A005F6668F9}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>